<commit_message>
feat(F-NAR-019): TREE-COL-020 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-020.xlsx
+++ b/stories/arbres/TREE-COL-020.xlsx
@@ -5008,17 +5008,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Nina prend le chat rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Et toi, tu as écouté la maîtresse. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer.</t>
+          <t>Nina prend le chat rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Toi, tu étais dans la classe. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina prend le &lt;emphasis level="moderate"&gt;chat&lt;/emphasis&gt; rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Et toi, tu as écouté la maîtresse. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina prend le &lt;emphasis level="moderate"&gt;chat&lt;/emphasis&gt; rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Toi, tu étais dans la classe. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Nina prend le &lt;emphasis&gt;chat&lt;/emphasis&gt; rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Et toi, tu as écouté la maîtresse. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer. [pause]</t>
+          <t>Nina prend le &lt;emphasis&gt;chat&lt;/emphasis&gt; rayé et le seau. Elle rejoint papa, près de la haie. Papa, Sarah a parlé trop près. Je t'écoute, et maman aussi. Elle a dit que le seau était à elle. Toi, tu étais dans la classe. Oui, après, mon ventre s'est serré. Merci de nous le dire, ici. Ils retournent vers Sarah. Le seau peut servir à deux. On essaie. Le chat rayé a une griffe de sable. Je suis prête à rentrer. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5157,7 +5157,7 @@
 enfant-f|Papa, Sarah a parlé trop près.
 papa|Je t'écoute, et maman aussi.
 enfant-f|Elle a dit que le seau était à elle.
-maman|Et toi, tu as écouté la maîtresse.
+maman|Toi, tu étais dans la classe.
 enfant-f|Oui, après, mon ventre s'est serré.
 papa|Merci de nous le dire, ici.
 narrateur|Ils retournent vers Sarah.
@@ -8787,17 +8787,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Nina descend avec le chat rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'ai écouté la maîtresse, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos.</t>
+          <t>Nina descend avec le chat rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'étais dans la classe, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina descend avec le &lt;emphasis level="moderate"&gt;chat&lt;/emphasis&gt; rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'ai écouté la maîtresse, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina descend avec le &lt;emphasis level="moderate"&gt;chat&lt;/emphasis&gt; rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'étais dans la classe, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nina descend avec le &lt;emphasis&gt;chat&lt;/emphasis&gt; rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'ai écouté la maîtresse, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos. [pause]</t>
+          <t>Nina descend avec le &lt;emphasis&gt;chat&lt;/emphasis&gt; rayé sous le bras. Elle rejoint le banc des parents. Le ballon reste en bas, pour Sarah. Qu'est-ce que tu n'as pas pu dire ? Sarah a parlé trop près, à l'école. Pendant la classe. Oui, j'étais dans la classe, puis ça. Merci, on tient la phrase, maintenant. Sarah arrive, le ballon contre elle. Nina t'a attendue en bas. On se dit au revoir ? Au revoir, Sarah. Le chat rayé a une goutte sur le dos. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8937,7 +8937,7 @@
 maman|Qu'est-ce que tu n'as pas pu dire ?
 enfant-f|Sarah a parlé trop près, à l'école.
 papa|Pendant la classe.
-enfant-f|Oui, j'ai écouté la maîtresse, puis ça.
+enfant-f|Oui, j'étais dans la classe, puis ça.
 maman|Merci, on tient la phrase, maintenant.
 narrateur|Sarah arrive, le ballon contre elle.
 papa|Nina t'a attendue en bas.
@@ -17476,7 +17476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17589,6 +17589,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>